<commit_message>
Added/Updated Features ( Period selection,  straight df processing,  facility name to title)
Changed period selection from date to only month year

Removed unnecessary writing of summary to file and reading it again (summary now processed straight from dataframes)

added Facility name to final summary title
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -31,7 +31,7 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
@@ -464,7 +464,7 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
     <col width="7" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
   </cols>
@@ -472,7 +472,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ART Monthly Summary Form As At April 2025</t>
+          <t>Holy Rosary Hospital ART Monthly Summary Form As At April 2025</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -601,28 +601,28 @@
         <v>0</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="R4" s="4" t="n"/>
     </row>
@@ -648,37 +648,37 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
         <v>1</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -859,7 +859,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -953,49 +953,49 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>9</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="K12" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="N12" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="L12" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>63</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>39</v>
-      </c>
       <c r="O12" s="4" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>425</v>
+        <v>411</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1009,49 +1009,49 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H13" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="I13" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="J13" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="K13" t="n">
-        <v>141</v>
+        <v>192</v>
       </c>
       <c r="L13" t="n">
-        <v>114</v>
+        <v>179</v>
       </c>
       <c r="M13" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="N13" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="O13" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="P13" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="Q13" t="n">
-        <v>751</v>
+        <v>847</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="R14" s="4" t="n"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16"/>
@@ -1176,7 +1176,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1207,16 +1207,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C19" t="n">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="D19" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>723</v>
+        <v>838</v>
       </c>
     </row>
     <row r="20">
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F20" s="4" t="n"/>
     </row>
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>727</v>
+        <v>838</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>200</v>
+        <v>298</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>350</v>
+        <v>644</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1349,7 +1349,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1368,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" s="4" t="n"/>
     </row>
@@ -1379,16 +1379,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>182</v>
+        <v>98</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>308</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30">
@@ -1398,16 +1398,16 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>382</v>
+        <v>396</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>660</v>
+        <v>831</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1422,7 +1422,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>DSD_Model</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>1175</v>
+        <v>1250</v>
       </c>
       <c r="C34" s="4" t="n"/>
     </row>
@@ -1449,21 +1449,21 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36"/>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>&gt;&gt;&gt; ART 5: Number of PLHIV on ART (who were on ART at the beginning of the reporting period or initiated treatment during the reporting period) and had no clinical contact since their last expected contact.</t>
+          <t>&gt;&gt;&gt; ART 5: Number of PLHIV on ART who had no clinical contact since their last expected contact.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1569,7 +1569,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
@@ -1599,7 +1599,7 @@
         <v>0</v>
       </c>
       <c r="Q39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -1630,13 +1630,13 @@
         <v>0</v>
       </c>
       <c r="I40" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="J40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="L40" s="4" t="n">
         <v>1</v>
@@ -1645,7 +1645,7 @@
         <v>1</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O40" s="4" t="n">
         <v>0</v>
@@ -1654,7 +1654,7 @@
         <v>1</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1710,7 +1710,7 @@
         <v/>
       </c>
       <c r="Q41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="Q44" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R44" s="4" t="n"/>
     </row>
@@ -1891,7 +1891,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1985,49 +1985,49 @@
         <v>0</v>
       </c>
       <c r="C48" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P48" s="4" t="n">
         <v>23</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>308</v>
+        <v>343</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2041,49 +2041,49 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G49" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H49" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="I49" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J49" t="n">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="K49" t="n">
-        <v>111</v>
+        <v>162</v>
       </c>
       <c r="L49" t="n">
-        <v>91</v>
+        <v>150</v>
       </c>
       <c r="M49" t="n">
-        <v>66</v>
+        <v>99</v>
       </c>
       <c r="N49" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="O49" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="P49" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="Q49" t="n">
-        <v>576</v>
+        <v>713</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="Q51" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52"/>
@@ -2208,7 +2208,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -2323,20 +2323,20 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
       </c>
       <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="n">
         <v>1</v>
       </c>
-      <c r="N55" t="n">
-        <v>0</v>
-      </c>
       <c r="O55" t="n">
         <v>0</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56">
@@ -2375,31 +2375,31 @@
         <v>0</v>
       </c>
       <c r="I56" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J56" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K56" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="L56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2455,7 +2455,7 @@
         <v/>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
@@ -2566,7 +2566,7 @@
         <v/>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
@@ -2636,7 +2636,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -2730,49 +2730,49 @@
         <v>0</v>
       </c>
       <c r="C64" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="I64" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J64" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="J64" s="4" t="n">
-        <v>23</v>
-      </c>
       <c r="K64" s="4" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="P64" s="4" t="n">
         <v>22</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>294</v>
+        <v>318</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2786,49 +2786,49 @@
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" t="n">
         <v>8</v>
-      </c>
-      <c r="E65" t="n">
-        <v>12</v>
-      </c>
-      <c r="F65" t="n">
-        <v>5</v>
       </c>
       <c r="G65" t="n">
         <v>10</v>
       </c>
       <c r="H65" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="I65" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="J65" t="n">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="K65" t="n">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="L65" t="n">
-        <v>87</v>
+        <v>143</v>
       </c>
       <c r="M65" t="n">
-        <v>63</v>
+        <v>97</v>
       </c>
       <c r="N65" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="O65" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="P65" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="Q65" t="n">
-        <v>551</v>
+        <v>681</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68"/>
@@ -2953,7 +2953,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -3068,20 +3068,20 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>
       </c>
       <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
         <v>1</v>
       </c>
-      <c r="N71" t="n">
-        <v>0</v>
-      </c>
       <c r="O71" t="n">
         <v>0</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
@@ -3120,14 +3120,14 @@
         <v>0</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K72" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="L72" s="4" t="n">
         <v>0</v>
       </c>
@@ -3138,13 +3138,13 @@
         <v>0</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3200,7 +3200,7 @@
         <v/>
       </c>
       <c r="Q73" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74">
@@ -3311,7 +3311,7 @@
         <v/>
       </c>
       <c r="Q75" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">

</xml_diff>

<commit_message>
Added baseline ART Line list data and ART8, 9 and 10
Baseline ART line list will be optional but recommended, it will be compared with current ART line list to know actual restarts

addded ART 8, 9 and 10
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R76"/>
+  <dimension ref="A1:R96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1036,10 +1036,10 @@
         <v>192</v>
       </c>
       <c r="L13" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="M13" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N13" t="n">
         <v>56</v>
@@ -2068,10 +2068,10 @@
         <v>162</v>
       </c>
       <c r="L49" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="M49" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="N49" t="n">
         <v>49</v>
@@ -2813,10 +2813,10 @@
         <v>156</v>
       </c>
       <c r="L65" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="M65" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="N65" t="n">
         <v>49</v>
@@ -3370,19 +3370,847 @@
       </c>
       <c r="R76" s="4" t="n"/>
     </row>
+    <row r="77"/>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>&gt;&gt;&gt; ART 8: Number of PLHIV who RESTARTED ART during the month</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>&lt;1</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>5-9</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>10-14</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>20-24</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>25-29</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>30-34</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>35-39</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>40-44</t>
+        </is>
+      </c>
+      <c r="L79" s="3" t="inlineStr">
+        <is>
+          <t>45-49</t>
+        </is>
+      </c>
+      <c r="M79" s="3" t="inlineStr">
+        <is>
+          <t>50-54</t>
+        </is>
+      </c>
+      <c r="N79" s="3" t="inlineStr">
+        <is>
+          <t>55-59</t>
+        </is>
+      </c>
+      <c r="O79" s="3" t="inlineStr">
+        <is>
+          <t>60-64</t>
+        </is>
+      </c>
+      <c r="P79" s="3" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="Q79" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82"/>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;&gt;&gt; ART 9: Number of PLHIV who were TRANSFERRED IN during the month </t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>&lt;1</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>5-9</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>10-14</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>20-24</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>25-29</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>30-34</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>35-39</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>40-44</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t>45-49</t>
+        </is>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>50-54</t>
+        </is>
+      </c>
+      <c r="N84" s="3" t="inlineStr">
+        <is>
+          <t>55-59</t>
+        </is>
+      </c>
+      <c r="O84" s="3" t="inlineStr">
+        <is>
+          <t>60-64</t>
+        </is>
+      </c>
+      <c r="P84" s="3" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="Q84" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" s="4" t="n"/>
+    </row>
+    <row r="87"/>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>&gt;&gt;&gt; ART 10: Number of PLHIV on ART (Including PMTCT) who were Clinically Screened for TB in HIV Treatment Settings - Newly initiated on ART</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>&lt;1</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>5-9</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>10-14</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>20-24</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>25-29</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>30-34</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>35-39</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>40-44</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>45-49</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>50-54</t>
+        </is>
+      </c>
+      <c r="N89" s="3" t="inlineStr">
+        <is>
+          <t>55-59</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="inlineStr">
+        <is>
+          <t>60-64</t>
+        </is>
+      </c>
+      <c r="P89" s="3" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="Q89" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92"/>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>&gt;&gt;&gt; ART 10: Number of PLHIV on ART (Including PMTCT) who were Clinically Screened for TB in HIV Treatment Settings - Previously on ART</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>&lt;1</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>5-9</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>10-14</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>15-19</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>20-24</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>25-29</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>30-34</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>35-39</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr">
+        <is>
+          <t>40-44</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t>45-49</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>50-54</t>
+        </is>
+      </c>
+      <c r="N94" s="3" t="inlineStr">
+        <is>
+          <t>55-59</t>
+        </is>
+      </c>
+      <c r="O94" s="3" t="inlineStr">
+        <is>
+          <t>60-64</t>
+        </is>
+      </c>
+      <c r="P94" s="3" t="inlineStr">
+        <is>
+          <t>65+</t>
+        </is>
+      </c>
+      <c r="Q94" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="n">
+        <v>5</v>
+      </c>
+      <c r="G95" t="n">
+        <v>5</v>
+      </c>
+      <c r="H95" t="n">
+        <v>3</v>
+      </c>
+      <c r="I95" t="n">
+        <v>6</v>
+      </c>
+      <c r="J95" t="n">
+        <v>11</v>
+      </c>
+      <c r="K95" t="n">
+        <v>13</v>
+      </c>
+      <c r="L95" t="n">
+        <v>20</v>
+      </c>
+      <c r="M95" t="n">
+        <v>11</v>
+      </c>
+      <c r="N95" t="n">
+        <v>12</v>
+      </c>
+      <c r="O95" t="n">
+        <v>9</v>
+      </c>
+      <c r="P95" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G96" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H96" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I96" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="J96" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K96" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="L96" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="M96" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="N96" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O96" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P96" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q96" s="4" t="n">
+        <v>229</v>
+      </c>
+      <c r="R96" s="4" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="15">
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A62:R62"/>
+    <mergeCell ref="A78:R78"/>
     <mergeCell ref="A53:R53"/>
     <mergeCell ref="A69:R69"/>
     <mergeCell ref="A2:R2"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="A10:R10"/>
     <mergeCell ref="A46:R46"/>
+    <mergeCell ref="A88:R88"/>
+    <mergeCell ref="A93:R93"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A37:R37"/>
     <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A83:R83"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Viral Load Indication Updated
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -2059,13 +2059,13 @@
         <v>25</v>
       </c>
       <c r="I49" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J49" t="n">
         <v>93</v>
       </c>
       <c r="K49" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L49" t="n">
         <v>149</v>
@@ -2083,7 +2083,7 @@
         <v>24</v>
       </c>
       <c r="Q49" t="n">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2375,13 +2375,13 @@
         <v>0</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L56" s="4" t="n">
         <v>0</v>
@@ -2399,7 +2399,7 @@
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2455,7 +2455,7 @@
         <v/>
       </c>
       <c r="Q57" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -2566,7 +2566,7 @@
         <v/>
       </c>
       <c r="Q59" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -2804,13 +2804,13 @@
         <v>21</v>
       </c>
       <c r="I65" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J65" t="n">
         <v>86</v>
       </c>
       <c r="K65" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="L65" t="n">
         <v>142</v>
@@ -2828,7 +2828,7 @@
         <v>24</v>
       </c>
       <c r="Q65" t="n">
-        <v>681</v>
+        <v>683</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -3120,13 +3120,13 @@
         <v>0</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L72" s="4" t="n">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3200,7 +3200,7 @@
         <v/>
       </c>
       <c r="Q73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -3311,7 +3311,7 @@
         <v/>
       </c>
       <c r="Q75" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">

</xml_diff>

<commit_message>
added option to read csv and more structured file load
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -464,8 +464,8 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -595,10 +595,10 @@
         <v>1</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>0</v>
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n"/>
     </row>
@@ -648,16 +648,16 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
         <v>3</v>
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -953,19 +953,19 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>17</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>29</v>
@@ -977,25 +977,25 @@
         <v>49</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>111</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>99</v>
+        <v>39</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>616</v>
+        <v>418</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1015,43 +1015,43 @@
         <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F13" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G13" t="n">
         <v>36</v>
       </c>
       <c r="H13" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I13" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J13" t="n">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K13" t="n">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="L13" t="n">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="M13" t="n">
-        <v>145</v>
+        <v>50</v>
       </c>
       <c r="N13" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>1246</v>
+        <v>958</v>
       </c>
     </row>
     <row r="14">
@@ -1210,13 +1210,13 @@
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>584</v>
+        <v>393</v>
       </c>
       <c r="D19" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E19" t="n">
-        <v>1220</v>
+        <v>937</v>
       </c>
     </row>
     <row r="20">
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F20" s="4" t="n"/>
     </row>
@@ -1268,13 +1268,13 @@
         <v>18</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>598</v>
+        <v>400</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>1229</v>
+        <v>942</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1323,13 +1323,13 @@
         <v>14</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>393</v>
+        <v>278</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>828</v>
+        <v>654</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1382,13 +1382,13 @@
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>176</v>
+        <v>103</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>364</v>
+        <v>257</v>
       </c>
     </row>
     <row r="30">
@@ -1401,13 +1401,13 @@
         <v>14</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>570</v>
+        <v>382</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1192</v>
+        <v>911</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1563,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
         <v>3</v>
@@ -1581,10 +1581,10 @@
         <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
@@ -1596,10 +1596,10 @@
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q39" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40">
@@ -1612,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" s="4" t="n">
         <v>0</v>
@@ -1627,10 +1627,10 @@
         <v>4</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J40" s="4" t="n">
         <v>6</v>
@@ -1642,19 +1642,19 @@
         <v>2</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N40" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O40" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1710,7 +1710,7 @@
         <v/>
       </c>
       <c r="Q41" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44">
@@ -1985,49 +1985,49 @@
         <v>0</v>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G48" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="G48" s="4" t="n">
-        <v>12</v>
-      </c>
       <c r="H48" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="P48" s="4" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>506</v>
+        <v>321</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2047,43 +2047,43 @@
         <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F49" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G49" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H49" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I49" t="n">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="J49" t="n">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="K49" t="n">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="L49" t="n">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="M49" t="n">
-        <v>130</v>
+        <v>43</v>
       </c>
       <c r="N49" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="O49" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>1043</v>
+        <v>718</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2730,49 +2730,49 @@
         <v>0</v>
       </c>
       <c r="C64" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I64" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="J64" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="J64" s="4" t="n">
-        <v>33</v>
-      </c>
       <c r="K64" s="4" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>82</v>
+        <v>32</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>461</v>
+        <v>292</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2792,43 +2792,43 @@
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F65" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G65" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H65" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I65" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="J65" t="n">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="K65" t="n">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="L65" t="n">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="M65" t="n">
-        <v>121</v>
+        <v>41</v>
       </c>
       <c r="N65" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="O65" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>970</v>
+        <v>663</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -3487,37 +3487,37 @@
         <v>0</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I80" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J80" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J80" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K80" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L80" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M80" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N80" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O80" s="4" t="n">
         <v>0</v>
       </c>
       <c r="P80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q80" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3543,25 +3543,25 @@
         <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H81" t="n">
         <v>1</v>
       </c>
       <c r="I81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K81" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L81" t="n">
         <v>3</v>
       </c>
       <c r="M81" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N81" t="n">
         <v>0</v>
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="82"/>
@@ -3693,7 +3693,7 @@
         <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H85" t="n">
         <v>0</v>
@@ -3702,10 +3702,10 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L85" t="n">
         <v>0</v>
@@ -3714,7 +3714,7 @@
         <v>0</v>
       </c>
       <c r="N85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O85" t="n">
         <v>0</v>
@@ -3723,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3754,13 +3754,13 @@
         <v>0</v>
       </c>
       <c r="I86" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J86" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K86" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L86" s="4" t="n">
         <v>0</v>
@@ -3778,7 +3778,7 @@
         <v>0</v>
       </c>
       <c r="Q86" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R86" s="4" t="n"/>
     </row>
@@ -3902,10 +3902,10 @@
         <v>1</v>
       </c>
       <c r="H90" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I90" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J90" s="4" t="n">
         <v>0</v>
@@ -3929,7 +3929,7 @@
         <v>0</v>
       </c>
       <c r="Q90" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R90" s="4" t="n"/>
     </row>
@@ -3955,16 +3955,16 @@
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H91" t="n">
         <v>2</v>
       </c>
       <c r="I91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K91" t="n">
         <v>3</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="92"/>
@@ -4093,49 +4093,49 @@
         <v>0</v>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D95" t="n">
         <v>3</v>
       </c>
       <c r="E95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G95" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H95" t="n">
         <v>7</v>
       </c>
       <c r="I95" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="J95" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="K95" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="L95" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="M95" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="N95" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="O95" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P95" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="Q95" t="n">
-        <v>188</v>
+        <v>91</v>
       </c>
     </row>
     <row r="96">
@@ -4154,43 +4154,43 @@
         <v>0</v>
       </c>
       <c r="E96" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G96" s="4" t="n">
         <v>10</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="N96" s="4" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="O96" s="4" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="P96" s="4" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="Q96" s="4" t="n">
-        <v>367</v>
+        <v>235</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
parse date function reverted to initial code
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -472,7 +472,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Immaculate Heart Hospital (Nkpor) ART Monthly Summary Form As At April 2025</t>
+          <t>Holy Rosary Hospital ART Monthly Summary Form As At April 2025</t>
         </is>
       </c>
     </row>
@@ -592,16 +592,16 @@
         <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>0</v>
@@ -610,7 +610,7 @@
         <v>1</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>0</v>
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R4" s="4" t="n"/>
     </row>
@@ -633,52 +633,52 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v/>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v/>
       </c>
       <c r="J5" t="n">
-        <v>3</v>
+        <v/>
       </c>
       <c r="K5" t="n">
-        <v>3</v>
+        <v/>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="Q5" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -733,7 +733,7 @@
         <v/>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R6" s="4" t="n"/>
     </row>
@@ -844,7 +844,7 @@
         <v/>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" s="4" t="n"/>
     </row>
@@ -953,38 +953,38 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F12" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="G12" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="H12" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>94</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>111</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>39</v>
-      </c>
       <c r="N12" s="4" t="n">
         <v>0</v>
       </c>
@@ -995,7 +995,7 @@
         <v>0</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>418</v>
+        <v>255</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1009,37 +1009,37 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="H13" t="n">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="I13" t="n">
-        <v>116</v>
+        <v>67</v>
       </c>
       <c r="J13" t="n">
+        <v>107</v>
+      </c>
+      <c r="K13" t="n">
+        <v>195</v>
+      </c>
+      <c r="L13" t="n">
         <v>177</v>
       </c>
-      <c r="K13" t="n">
-        <v>257</v>
-      </c>
-      <c r="L13" t="n">
-        <v>197</v>
-      </c>
       <c r="M13" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -1051,7 +1051,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>958</v>
+        <v>660</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="R14" s="4" t="n"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="Q15" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16"/>
@@ -1207,16 +1207,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C19" t="n">
-        <v>393</v>
+        <v>244</v>
       </c>
       <c r="D19" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>937</v>
+        <v>651</v>
       </c>
     </row>
     <row r="20">
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F20" s="4" t="n"/>
     </row>
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>400</v>
+        <v>244</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>942</v>
+        <v>651</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>278</v>
+        <v>183</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>654</v>
+        <v>504</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1343,7 +1343,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -1382,13 +1382,13 @@
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>103</v>
+        <v>58</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>257</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30">
@@ -1398,16 +1398,16 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>382</v>
+        <v>241</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>911</v>
+        <v>644</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>1599</v>
+        <v>1250</v>
       </c>
       <c r="C34" s="4" t="n"/>
     </row>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>263</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36"/>
@@ -1560,46 +1560,46 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
         <v>1</v>
       </c>
-      <c r="E39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" t="n">
-        <v>3</v>
-      </c>
-      <c r="G39" t="n">
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
         <v>2</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" t="n">
-        <v>2</v>
-      </c>
-      <c r="K39" t="n">
-        <v>3</v>
-      </c>
-      <c r="L39" t="n">
-        <v>3</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="40">
@@ -1621,40 +1621,40 @@
         <v>0</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I40" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J40" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K40" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L40" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M40" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="4" t="n">
-        <v>24</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1765,7 +1765,7 @@
         <v/>
       </c>
       <c r="Q42" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R42" s="4" t="n"/>
     </row>
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="Q44" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R44" s="4" t="n"/>
     </row>
@@ -1985,37 +1985,37 @@
         <v>0</v>
       </c>
       <c r="C48" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="N48" s="4" t="n">
         <v>0</v>
@@ -2027,7 +2027,7 @@
         <v>0</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>321</v>
+        <v>203</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2041,37 +2041,37 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G49" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="H49" t="n">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="I49" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="J49" t="n">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="K49" t="n">
-        <v>196</v>
+        <v>162</v>
       </c>
       <c r="L49" t="n">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="M49" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="N49" t="n">
         <v>0</v>
@@ -2083,7 +2083,7 @@
         <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>718</v>
+        <v>533</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="Q51" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52"/>
@@ -2320,16 +2320,16 @@
         <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J55" t="n">
         <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M55" t="n">
         <v>0</v>
@@ -2344,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
@@ -2372,34 +2372,34 @@
         <v>0</v>
       </c>
       <c r="H56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="4" t="n">
+      <c r="N56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="K56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q56" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2730,37 +2730,37 @@
         <v>0</v>
       </c>
       <c r="C64" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F64" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H64" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G64" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="H64" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="I64" s="4" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="N64" s="4" t="n">
         <v>0</v>
@@ -2772,7 +2772,7 @@
         <v>0</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>292</v>
+        <v>184</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2786,37 +2786,37 @@
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D65" t="n">
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F65" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G65" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="H65" t="n">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="I65" t="n">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="J65" t="n">
-        <v>117</v>
+        <v>83</v>
       </c>
       <c r="K65" t="n">
-        <v>179</v>
+        <v>154</v>
       </c>
       <c r="L65" t="n">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="M65" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="N65" t="n">
         <v>0</v>
@@ -2828,7 +2828,7 @@
         <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>663</v>
+        <v>502</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="Q67" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68"/>
@@ -3068,13 +3068,13 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M71" t="n">
         <v>0</v>
@@ -3089,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I72" s="4" t="n">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3487,22 +3487,22 @@
         <v>0</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I80" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M80" s="4" t="n">
         <v>0</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="Q80" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3543,37 +3543,37 @@
         <v>0</v>
       </c>
       <c r="G81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
         <v>2</v>
-      </c>
-      <c r="H81" t="n">
-        <v>1</v>
-      </c>
-      <c r="I81" t="n">
-        <v>2</v>
-      </c>
-      <c r="J81" t="n">
-        <v>4</v>
-      </c>
-      <c r="K81" t="n">
-        <v>6</v>
-      </c>
-      <c r="L81" t="n">
-        <v>3</v>
-      </c>
-      <c r="M81" t="n">
-        <v>0</v>
-      </c>
-      <c r="N81" t="n">
-        <v>0</v>
-      </c>
-      <c r="O81" t="n">
-        <v>0</v>
-      </c>
-      <c r="P81" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q81" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="82"/>
@@ -3708,7 +3708,7 @@
         <v>0</v>
       </c>
       <c r="L85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M85" t="n">
         <v>0</v>
@@ -3723,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -3899,16 +3899,16 @@
         <v>0</v>
       </c>
       <c r="G90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="H90" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I90" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J90" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="K90" s="4" t="n">
         <v>0</v>
@@ -3917,7 +3917,7 @@
         <v>1</v>
       </c>
       <c r="M90" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N90" s="4" t="n">
         <v>0</v>
@@ -3929,7 +3929,7 @@
         <v>0</v>
       </c>
       <c r="Q90" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R90" s="4" t="n"/>
     </row>
@@ -3955,19 +3955,19 @@
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H91" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K91" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L91" t="n">
         <v>0</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92"/>
@@ -4096,34 +4096,34 @@
         <v>0</v>
       </c>
       <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>5</v>
+      </c>
+      <c r="G95" t="n">
+        <v>1</v>
+      </c>
+      <c r="H95" t="n">
         <v>3</v>
       </c>
-      <c r="E95" t="n">
-        <v>3</v>
-      </c>
-      <c r="F95" t="n">
-        <v>3</v>
-      </c>
-      <c r="G95" t="n">
-        <v>3</v>
-      </c>
-      <c r="H95" t="n">
-        <v>7</v>
-      </c>
       <c r="I95" t="n">
+        <v>5</v>
+      </c>
+      <c r="J95" t="n">
+        <v>6</v>
+      </c>
+      <c r="K95" t="n">
         <v>9</v>
       </c>
-      <c r="J95" t="n">
-        <v>16</v>
-      </c>
-      <c r="K95" t="n">
-        <v>17</v>
-      </c>
       <c r="L95" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="M95" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N95" t="n">
         <v>0</v>
@@ -4135,7 +4135,7 @@
         <v>0</v>
       </c>
       <c r="Q95" t="n">
-        <v>91</v>
+        <v>44</v>
       </c>
     </row>
     <row r="96">
@@ -4154,31 +4154,31 @@
         <v>0</v>
       </c>
       <c r="E96" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="N96" s="4" t="n">
         <v>0</v>
@@ -4190,7 +4190,7 @@
         <v>0</v>
       </c>
       <c r="Q96" s="4" t="n">
-        <v>235</v>
+        <v>118</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
reverted dateparse and esnured datetime format
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -464,7 +464,7 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
     <col width="7" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
   </cols>
@@ -633,52 +633,52 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -962,40 +962,40 @@
         <v>9</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>14</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>50</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>18</v>
+        <v>64</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>255</v>
+        <v>411</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1012,46 +1012,46 @@
         <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
         <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H13" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I13" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="J13" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="K13" t="n">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="L13" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="M13" t="n">
-        <v>41</v>
+        <v>113</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="Q13" t="n">
-        <v>660</v>
+        <v>847</v>
       </c>
     </row>
     <row r="14">
@@ -1210,13 +1210,13 @@
         <v>11</v>
       </c>
       <c r="C19" t="n">
-        <v>244</v>
+        <v>400</v>
       </c>
       <c r="D19" t="n">
         <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>651</v>
+        <v>838</v>
       </c>
     </row>
     <row r="20">
@@ -1268,13 +1268,13 @@
         <v>11</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>244</v>
+        <v>400</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>9</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>651</v>
+        <v>838</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1323,13 +1323,13 @@
         <v>11</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>183</v>
+        <v>298</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>9</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>504</v>
+        <v>644</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1382,13 +1382,13 @@
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>140</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30">
@@ -1401,13 +1401,13 @@
         <v>11</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>241</v>
+        <v>396</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>9</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>644</v>
+        <v>831</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J40" s="4" t="n">
         <v>0</v>
@@ -1639,10 +1639,10 @@
         <v>1</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N40" s="4" t="n">
         <v>0</v>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1710,7 +1710,7 @@
         <v/>
       </c>
       <c r="Q41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44">
@@ -1991,43 +1991,43 @@
         <v>1</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H48" s="4" t="n">
         <v>9</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L48" s="4" t="n">
         <v>64</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="P48" s="4" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>203</v>
+        <v>344</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2044,46 +2044,46 @@
         <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
         <v>11</v>
       </c>
       <c r="G49" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H49" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I49" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="J49" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K49" t="n">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="L49" t="n">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="M49" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="O49" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Q49" t="n">
-        <v>533</v>
+        <v>716</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="Q51" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52"/>
@@ -2335,7 +2335,7 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O55" t="n">
         <v>0</v>
@@ -2344,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56">
@@ -2375,7 +2375,7 @@
         <v>0</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J56" s="4" t="n">
         <v>0</v>
@@ -2393,13 +2393,13 @@
         <v>0</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2736,43 +2736,43 @@
         <v>1</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H64" s="4" t="n">
         <v>8</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="L64" s="4" t="n">
         <v>58</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>184</v>
+        <v>319</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2789,46 +2789,46 @@
         <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
         <v>8</v>
       </c>
       <c r="G65" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H65" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I65" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="J65" t="n">
         <v>83</v>
       </c>
       <c r="K65" t="n">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="L65" t="n">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="M65" t="n">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="N65" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="O65" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Q65" t="n">
-        <v>502</v>
+        <v>684</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="Q67" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68"/>
@@ -3080,7 +3080,7 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O71" t="n">
         <v>0</v>
@@ -3089,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
@@ -3138,13 +3138,13 @@
         <v>0</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3505,7 +3505,7 @@
         <v>0</v>
       </c>
       <c r="M80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N80" s="4" t="n">
         <v>0</v>
@@ -3517,7 +3517,7 @@
         <v>0</v>
       </c>
       <c r="Q80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3543,7 +3543,7 @@
         <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H81" t="n">
         <v>0</v>
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82"/>
@@ -3708,7 +3708,7 @@
         <v>0</v>
       </c>
       <c r="L85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M85" t="n">
         <v>0</v>
@@ -3723,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3955,7 +3955,7 @@
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92"/>
@@ -4099,43 +4099,43 @@
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F95" t="n">
         <v>5</v>
       </c>
       <c r="G95" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H95" t="n">
         <v>3</v>
       </c>
       <c r="I95" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J95" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K95" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L95" t="n">
+        <v>20</v>
+      </c>
+      <c r="M95" t="n">
+        <v>11</v>
+      </c>
+      <c r="N95" t="n">
         <v>13</v>
       </c>
-      <c r="M95" t="n">
-        <v>0</v>
-      </c>
-      <c r="N95" t="n">
-        <v>0</v>
-      </c>
       <c r="O95" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P95" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q95" t="n">
-        <v>44</v>
+        <v>106</v>
       </c>
     </row>
     <row r="96">
@@ -4148,7 +4148,7 @@
         <v>0</v>
       </c>
       <c r="C96" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D96" s="4" t="n">
         <v>0</v>
@@ -4157,40 +4157,40 @@
         <v>0</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="N96" s="4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O96" s="4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P96" s="4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q96" s="4" t="n">
-        <v>118</v>
+        <v>229</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
updated parse_date function to remove out of bound dates
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -464,15 +464,15 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Holy Rosary Hospital ART Monthly Summary Form As At April 2025</t>
+          <t>Nnamdi Azikiwe University Teaching Hospital ART Monthly Summary Form As At April 2025</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>1</v>
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R4" s="4" t="n"/>
     </row>
@@ -648,7 +648,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -657,7 +657,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -675,10 +675,10 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -953,49 +953,49 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>50</v>
+        <v>88</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>64</v>
+        <v>234</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>56</v>
+        <v>220</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>27</v>
+        <v>170</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>25</v>
+        <v>182</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>411</v>
+        <v>1307</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1009,49 +1009,49 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="G13" t="n">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="H13" t="n">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="I13" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="J13" t="n">
-        <v>104</v>
+        <v>172</v>
       </c>
       <c r="K13" t="n">
-        <v>197</v>
+        <v>382</v>
       </c>
       <c r="L13" t="n">
-        <v>178</v>
+        <v>581</v>
       </c>
       <c r="M13" t="n">
-        <v>113</v>
+        <v>523</v>
       </c>
       <c r="N13" t="n">
-        <v>55</v>
+        <v>303</v>
       </c>
       <c r="O13" t="n">
-        <v>28</v>
+        <v>189</v>
       </c>
       <c r="P13" t="n">
-        <v>29</v>
+        <v>184</v>
       </c>
       <c r="Q13" t="n">
-        <v>847</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="R14" s="4" t="n"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="Q15" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16"/>
@@ -1207,16 +1207,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C19" t="n">
-        <v>400</v>
+        <v>1069</v>
       </c>
       <c r="D19" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E19" t="n">
-        <v>838</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="20">
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>0</v>
+        <v>212</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="F20" s="4" t="n"/>
     </row>
@@ -1249,13 +1249,13 @@
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>400</v>
+        <v>1286</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>838</v>
+        <v>2587</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>298</v>
+        <v>644</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>644</v>
+        <v>1224</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1343,13 +1343,13 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -1362,10 +1362,10 @@
         <v>0</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>0</v>
@@ -1379,16 +1379,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>98</v>
+        <v>594</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>187</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="30">
@@ -1398,16 +1398,16 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>396</v>
+        <v>1240</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>831</v>
+        <v>2525</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>1250</v>
+        <v>3809</v>
       </c>
       <c r="C34" s="4" t="n"/>
     </row>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>8</v>
+        <v/>
       </c>
     </row>
     <row r="36"/>
@@ -1566,40 +1566,40 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q39" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40">
@@ -1624,7 +1624,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H40" s="4" t="n">
         <v>0</v>
@@ -1633,28 +1633,28 @@
         <v>3</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O40" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1710,7 +1710,7 @@
         <v/>
       </c>
       <c r="Q41" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42">
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="Q44" s="4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R44" s="4" t="n"/>
     </row>
@@ -1988,46 +1988,46 @@
         <v>1</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>52</v>
+        <v>197</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>45</v>
+        <v>180</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>26</v>
+        <v>150</v>
       </c>
       <c r="P48" s="4" t="n">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>344</v>
+        <v>1079</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2041,49 +2041,49 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F49" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="G49" t="n">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="H49" t="n">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="I49" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="J49" t="n">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="K49" t="n">
+        <v>324</v>
+      </c>
+      <c r="L49" t="n">
+        <v>501</v>
+      </c>
+      <c r="M49" t="n">
+        <v>460</v>
+      </c>
+      <c r="N49" t="n">
+        <v>269</v>
+      </c>
+      <c r="O49" t="n">
         <v>169</v>
       </c>
-      <c r="L49" t="n">
-        <v>148</v>
-      </c>
-      <c r="M49" t="n">
-        <v>95</v>
-      </c>
-      <c r="N49" t="n">
-        <v>49</v>
-      </c>
-      <c r="O49" t="n">
-        <v>25</v>
-      </c>
       <c r="P49" t="n">
-        <v>24</v>
+        <v>153</v>
       </c>
       <c r="Q49" t="n">
-        <v>716</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2323,10 +2323,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
@@ -2338,10 +2338,10 @@
         <v>1</v>
       </c>
       <c r="O55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q55" t="n">
         <v>4</v>
@@ -2375,31 +2375,31 @@
         <v>0</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N56" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2455,7 +2455,7 @@
         <v/>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -2566,7 +2566,7 @@
         <v/>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -2733,46 +2733,46 @@
         <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="J64" s="4" t="n">
         <v>28</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>50</v>
+        <v>193</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>44</v>
+        <v>171</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>22</v>
+        <v>155</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>319</v>
+        <v>1032</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2786,49 +2786,49 @@
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F65" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="G65" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="H65" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="I65" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J65" t="n">
-        <v>83</v>
+        <v>139</v>
       </c>
       <c r="K65" t="n">
-        <v>162</v>
+        <v>313</v>
       </c>
       <c r="L65" t="n">
-        <v>142</v>
+        <v>487</v>
       </c>
       <c r="M65" t="n">
-        <v>93</v>
+        <v>451</v>
       </c>
       <c r="N65" t="n">
-        <v>49</v>
+        <v>267</v>
       </c>
       <c r="O65" t="n">
-        <v>25</v>
+        <v>166</v>
       </c>
       <c r="P65" t="n">
-        <v>24</v>
+        <v>151</v>
       </c>
       <c r="Q65" t="n">
-        <v>684</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="66">
@@ -3068,7 +3068,7 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" t="n">
         <v>1</v>
@@ -3083,13 +3083,13 @@
         <v>1</v>
       </c>
       <c r="O71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q71" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72">
@@ -3126,25 +3126,25 @@
         <v>0</v>
       </c>
       <c r="K72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="N72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3481,13 +3481,13 @@
         <v>0</v>
       </c>
       <c r="E80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H80" s="4" t="n">
         <v>0</v>
@@ -3499,25 +3499,25 @@
         <v>0</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L80" s="4" t="n">
         <v>0</v>
       </c>
       <c r="M80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N80" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P80" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q80" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3534,46 +3534,46 @@
         <v>0</v>
       </c>
       <c r="D81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L81" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M81" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="82"/>
@@ -3708,7 +3708,7 @@
         <v>0</v>
       </c>
       <c r="L85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M85" t="n">
         <v>0</v>
@@ -3720,10 +3720,10 @@
         <v>0</v>
       </c>
       <c r="P85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q85" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
@@ -3911,7 +3911,7 @@
         <v>1</v>
       </c>
       <c r="K90" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L90" s="4" t="n">
         <v>1</v>
@@ -3929,7 +3929,7 @@
         <v>0</v>
       </c>
       <c r="Q90" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R90" s="4" t="n"/>
     </row>
@@ -3955,7 +3955,7 @@
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
@@ -3964,7 +3964,7 @@
         <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -3982,10 +3982,10 @@
         <v>0</v>
       </c>
       <c r="P91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92"/>
@@ -4096,46 +4096,46 @@
         <v>0</v>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F95" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G95" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H95" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I95" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J95" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K95" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L95" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M95" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="N95" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="O95" t="n">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="P95" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="Q95" t="n">
-        <v>106</v>
+        <v>281</v>
       </c>
     </row>
     <row r="96">
@@ -4148,49 +4148,49 @@
         <v>0</v>
       </c>
       <c r="C96" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E96" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>47</v>
+        <v>137</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>41</v>
+        <v>123</v>
       </c>
       <c r="N96" s="4" t="n">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="O96" s="4" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="P96" s="4" t="n">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="Q96" s="4" t="n">
-        <v>229</v>
+        <v>618</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
updated VL Indication and added description for a single facility file upload
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ART MSF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ART MSF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,15 +464,15 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Nnamdi Azikiwe University Teaching Hospital ART Monthly Summary Form As At April 2025</t>
+          <t>Holy Rosary Hospital ART Monthly Summary Form As At April 2025</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>1</v>
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R4" s="4" t="n"/>
     </row>
@@ -648,7 +648,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -657,28 +657,28 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
         <v>1</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -953,49 +953,49 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>145</v>
+        <v>75</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>234</v>
+        <v>64</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>220</v>
+        <v>56</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>170</v>
+        <v>27</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>182</v>
+        <v>25</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1307</v>
+        <v>411</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1009,49 +1009,49 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="H13" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="I13" t="n">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="J13" t="n">
-        <v>172</v>
+        <v>104</v>
       </c>
       <c r="K13" t="n">
-        <v>382</v>
+        <v>197</v>
       </c>
       <c r="L13" t="n">
-        <v>581</v>
+        <v>178</v>
       </c>
       <c r="M13" t="n">
-        <v>523</v>
+        <v>113</v>
       </c>
       <c r="N13" t="n">
-        <v>303</v>
+        <v>55</v>
       </c>
       <c r="O13" t="n">
-        <v>189</v>
+        <v>28</v>
       </c>
       <c r="P13" t="n">
-        <v>184</v>
+        <v>29</v>
       </c>
       <c r="Q13" t="n">
-        <v>2617</v>
+        <v>847</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R14" s="4" t="n"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="Q15" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16"/>
@@ -1207,16 +1207,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C19" t="n">
-        <v>1069</v>
+        <v>400</v>
       </c>
       <c r="D19" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>2224</v>
+        <v>838</v>
       </c>
     </row>
     <row r="20">
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>212</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>360</v>
+        <v>0</v>
       </c>
       <c r="F20" s="4" t="n"/>
     </row>
@@ -1249,13 +1249,13 @@
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1286</v>
+        <v>400</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>2587</v>
+        <v>838</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C26" s="4" t="n">
+        <v>298</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" s="4" t="n">
         <v>644</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>1224</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1343,13 +1343,13 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1362,10 +1362,10 @@
         <v>0</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>0</v>
@@ -1379,16 +1379,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>594</v>
+        <v>98</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>1299</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30">
@@ -1398,16 +1398,16 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1240</v>
+        <v>396</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>2525</v>
+        <v>831</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>3809</v>
+        <v>1250</v>
       </c>
       <c r="C34" s="4" t="n"/>
     </row>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v/>
+        <v>8</v>
       </c>
     </row>
     <row r="36"/>
@@ -1566,40 +1566,40 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
         <v>1</v>
       </c>
-      <c r="G39" t="n">
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
         <v>1</v>
       </c>
-      <c r="H39" t="n">
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
         <v>2</v>
-      </c>
-      <c r="I39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J39" t="n">
-        <v>0</v>
-      </c>
-      <c r="K39" t="n">
-        <v>1</v>
-      </c>
-      <c r="L39" t="n">
-        <v>2</v>
-      </c>
-      <c r="M39" t="n">
-        <v>1</v>
-      </c>
-      <c r="N39" t="n">
-        <v>7</v>
-      </c>
-      <c r="O39" t="n">
-        <v>1</v>
-      </c>
-      <c r="P39" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>21</v>
       </c>
     </row>
     <row r="40">
@@ -1624,7 +1624,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H40" s="4" t="n">
         <v>0</v>
@@ -1633,28 +1633,28 @@
         <v>3</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1710,7 +1710,7 @@
         <v/>
       </c>
       <c r="Q41" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="Q44" s="4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R44" s="4" t="n"/>
     </row>
@@ -1988,46 +1988,46 @@
         <v>1</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>111</v>
+        <v>64</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>197</v>
+        <v>52</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>180</v>
+        <v>45</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>150</v>
+        <v>26</v>
       </c>
       <c r="P48" s="4" t="n">
-        <v>160</v>
+        <v>23</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>1079</v>
+        <v>344</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2041,49 +2041,49 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="G49" t="n">
+        <v>13</v>
+      </c>
+      <c r="H49" t="n">
+        <v>25</v>
+      </c>
+      <c r="I49" t="n">
+        <v>61</v>
+      </c>
+      <c r="J49" t="n">
+        <v>90</v>
+      </c>
+      <c r="K49" t="n">
+        <v>169</v>
+      </c>
+      <c r="L49" t="n">
+        <v>148</v>
+      </c>
+      <c r="M49" t="n">
+        <v>95</v>
+      </c>
+      <c r="N49" t="n">
         <v>49</v>
       </c>
-      <c r="H49" t="n">
-        <v>56</v>
-      </c>
-      <c r="I49" t="n">
-        <v>66</v>
-      </c>
-      <c r="J49" t="n">
-        <v>142</v>
-      </c>
-      <c r="K49" t="n">
-        <v>324</v>
-      </c>
-      <c r="L49" t="n">
-        <v>501</v>
-      </c>
-      <c r="M49" t="n">
-        <v>460</v>
-      </c>
-      <c r="N49" t="n">
-        <v>269</v>
-      </c>
       <c r="O49" t="n">
-        <v>169</v>
+        <v>25</v>
       </c>
       <c r="P49" t="n">
-        <v>153</v>
+        <v>24</v>
       </c>
       <c r="Q49" t="n">
-        <v>2242</v>
+        <v>716</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2323,10 +2323,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
@@ -2338,10 +2338,10 @@
         <v>1</v>
       </c>
       <c r="O55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q55" t="n">
         <v>4</v>
@@ -2375,31 +2375,31 @@
         <v>0</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L56" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M56" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="N56" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2455,7 +2455,7 @@
         <v/>
       </c>
       <c r="Q57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -2566,7 +2566,7 @@
         <v/>
       </c>
       <c r="Q59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -2733,46 +2733,46 @@
         <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="J64" s="4" t="n">
         <v>28</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>193</v>
+        <v>50</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>171</v>
+        <v>44</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>146</v>
+        <v>24</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>155</v>
+        <v>22</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>1032</v>
+        <v>319</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2786,49 +2786,49 @@
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" t="n">
+        <v>8</v>
+      </c>
+      <c r="G65" t="n">
         <v>11</v>
       </c>
-      <c r="F65" t="n">
-        <v>28</v>
-      </c>
-      <c r="G65" t="n">
-        <v>45</v>
-      </c>
       <c r="H65" t="n">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="I65" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J65" t="n">
-        <v>139</v>
+        <v>83</v>
       </c>
       <c r="K65" t="n">
-        <v>313</v>
+        <v>162</v>
       </c>
       <c r="L65" t="n">
-        <v>487</v>
+        <v>142</v>
       </c>
       <c r="M65" t="n">
-        <v>451</v>
+        <v>93</v>
       </c>
       <c r="N65" t="n">
-        <v>267</v>
+        <v>49</v>
       </c>
       <c r="O65" t="n">
-        <v>166</v>
+        <v>25</v>
       </c>
       <c r="P65" t="n">
-        <v>151</v>
+        <v>24</v>
       </c>
       <c r="Q65" t="n">
-        <v>2181</v>
+        <v>684</v>
       </c>
     </row>
     <row r="66">
@@ -3068,7 +3068,7 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K71" t="n">
         <v>1</v>
@@ -3083,13 +3083,13 @@
         <v>1</v>
       </c>
       <c r="O71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
@@ -3126,25 +3126,25 @@
         <v>0</v>
       </c>
       <c r="K72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L72" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M72" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N72" s="4" t="n">
+      <c r="P72" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="O72" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P72" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q72" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3481,43 +3481,43 @@
         <v>0</v>
       </c>
       <c r="E80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F80" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G80" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H80" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I80" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J80" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K80" s="4" t="n">
+      <c r="N80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="L80" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M80" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N80" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O80" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P80" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q80" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3534,46 +3534,46 @@
         <v>0</v>
       </c>
       <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
         <v>1</v>
       </c>
-      <c r="E81" t="n">
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
         <v>2</v>
-      </c>
-      <c r="F81" t="n">
-        <v>1</v>
-      </c>
-      <c r="G81" t="n">
-        <v>2</v>
-      </c>
-      <c r="H81" t="n">
-        <v>1</v>
-      </c>
-      <c r="I81" t="n">
-        <v>2</v>
-      </c>
-      <c r="J81" t="n">
-        <v>4</v>
-      </c>
-      <c r="K81" t="n">
-        <v>2</v>
-      </c>
-      <c r="L81" t="n">
-        <v>4</v>
-      </c>
-      <c r="M81" t="n">
-        <v>4</v>
-      </c>
-      <c r="N81" t="n">
-        <v>1</v>
-      </c>
-      <c r="O81" t="n">
-        <v>1</v>
-      </c>
-      <c r="P81" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q81" t="n">
-        <v>26</v>
       </c>
     </row>
     <row r="82"/>
@@ -3708,7 +3708,7 @@
         <v>0</v>
       </c>
       <c r="L85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M85" t="n">
         <v>0</v>
@@ -3720,10 +3720,10 @@
         <v>0</v>
       </c>
       <c r="P85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3911,7 +3911,7 @@
         <v>1</v>
       </c>
       <c r="K90" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L90" s="4" t="n">
         <v>1</v>
@@ -3929,7 +3929,7 @@
         <v>0</v>
       </c>
       <c r="Q90" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R90" s="4" t="n"/>
     </row>
@@ -3955,7 +3955,7 @@
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
@@ -3964,28 +3964,28 @@
         <v>0</v>
       </c>
       <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="n">
         <v>1</v>
-      </c>
-      <c r="K91" t="n">
-        <v>0</v>
-      </c>
-      <c r="L91" t="n">
-        <v>0</v>
-      </c>
-      <c r="M91" t="n">
-        <v>0</v>
-      </c>
-      <c r="N91" t="n">
-        <v>0</v>
-      </c>
-      <c r="O91" t="n">
-        <v>0</v>
-      </c>
-      <c r="P91" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q91" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="92"/>
@@ -4096,46 +4096,46 @@
         <v>0</v>
       </c>
       <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="n">
+        <v>5</v>
+      </c>
+      <c r="G95" t="n">
+        <v>5</v>
+      </c>
+      <c r="H95" t="n">
         <v>3</v>
       </c>
-      <c r="E95" t="n">
-        <v>4</v>
-      </c>
-      <c r="F95" t="n">
+      <c r="I95" t="n">
+        <v>6</v>
+      </c>
+      <c r="J95" t="n">
+        <v>11</v>
+      </c>
+      <c r="K95" t="n">
         <v>13</v>
       </c>
-      <c r="G95" t="n">
-        <v>17</v>
-      </c>
-      <c r="H95" t="n">
-        <v>15</v>
-      </c>
-      <c r="I95" t="n">
-        <v>9</v>
-      </c>
-      <c r="J95" t="n">
-        <v>10</v>
-      </c>
-      <c r="K95" t="n">
-        <v>12</v>
-      </c>
       <c r="L95" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="M95" t="n">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="N95" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="O95" t="n">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="P95" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="Q95" t="n">
-        <v>281</v>
+        <v>106</v>
       </c>
     </row>
     <row r="96">
@@ -4148,49 +4148,49 @@
         <v>0</v>
       </c>
       <c r="C96" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D96" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G96" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H96" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F96" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G96" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="H96" s="4" t="n">
-        <v>18</v>
-      </c>
       <c r="I96" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>137</v>
+        <v>47</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>123</v>
+        <v>41</v>
       </c>
       <c r="N96" s="4" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="O96" s="4" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="P96" s="4" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="Q96" s="4" t="n">
-        <v>618</v>
+        <v>229</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
applied use col and try & except block
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -464,15 +464,15 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Holy Rosary Hospital ART Monthly Summary Form As At April 2025</t>
+          <t>Onitsha General Hospital ART Monthly Summary Form As At April 2025</t>
         </is>
       </c>
     </row>
@@ -592,10 +592,10 @@
         <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>0</v>
@@ -604,14 +604,14 @@
         <v>1</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="N4" s="4" t="n">
         <v>0</v>
       </c>
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R4" s="4" t="n"/>
     </row>
@@ -642,34 +642,34 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -733,7 +733,7 @@
         <v/>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" s="4" t="n"/>
     </row>
@@ -953,49 +953,49 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>24</v>
+        <v>106</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>41</v>
+        <v>134</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>75</v>
+        <v>154</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>64</v>
+        <v>216</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>56</v>
+        <v>189</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>27</v>
+        <v>107</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>411</v>
+        <v>1425</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1012,46 +1012,46 @@
         <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="G13" t="n">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="H13" t="n">
-        <v>31</v>
+        <v>134</v>
       </c>
       <c r="I13" t="n">
-        <v>71</v>
+        <v>191</v>
       </c>
       <c r="J13" t="n">
-        <v>104</v>
+        <v>314</v>
       </c>
       <c r="K13" t="n">
-        <v>197</v>
+        <v>524</v>
       </c>
       <c r="L13" t="n">
-        <v>178</v>
+        <v>560</v>
       </c>
       <c r="M13" t="n">
-        <v>113</v>
+        <v>469</v>
       </c>
       <c r="N13" t="n">
-        <v>55</v>
+        <v>247</v>
       </c>
       <c r="O13" t="n">
-        <v>28</v>
+        <v>146</v>
       </c>
       <c r="P13" t="n">
-        <v>29</v>
+        <v>138</v>
       </c>
       <c r="Q13" t="n">
-        <v>847</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="R14" s="4" t="n"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="Q15" t="n">
-        <v>16</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16"/>
@@ -1207,16 +1207,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="C19" t="n">
-        <v>400</v>
+        <v>1369</v>
       </c>
       <c r="D19" t="n">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="E19" t="n">
-        <v>838</v>
+        <v>2803</v>
       </c>
     </row>
     <row r="20">
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F20" s="4" t="n"/>
     </row>
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>400</v>
+        <v>1390</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>838</v>
+        <v>2835</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>298</v>
+        <v>752</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>644</v>
+        <v>1573</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1343,13 +1343,13 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28">
@@ -1379,16 +1379,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C29" t="n">
-        <v>98</v>
+        <v>443</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E29" t="n">
-        <v>187</v>
+        <v>952</v>
       </c>
     </row>
     <row r="30">
@@ -1398,16 +1398,16 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>396</v>
+        <v>1235</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>831</v>
+        <v>2594</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>1250</v>
+        <v>4002</v>
       </c>
       <c r="C34" s="4" t="n"/>
     </row>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>8</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36"/>
@@ -1572,22 +1572,22 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
         <v>1</v>
       </c>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="n">
-        <v>0</v>
-      </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -1596,10 +1596,10 @@
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q39" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -1630,31 +1630,31 @@
         <v>0</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O40" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1710,7 +1710,7 @@
         <v/>
       </c>
       <c r="Q41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
@@ -1765,7 +1765,7 @@
         <v/>
       </c>
       <c r="Q42" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R42" s="4" t="n"/>
     </row>
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="Q44" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R44" s="4" t="n"/>
     </row>
@@ -1985,49 +1985,49 @@
         <v>0</v>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>33</v>
+        <v>103</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>52</v>
+        <v>180</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>45</v>
+        <v>166</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>26</v>
+        <v>97</v>
       </c>
       <c r="P48" s="4" t="n">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>344</v>
+        <v>1184</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2041,49 +2041,49 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F49" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="G49" t="n">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="H49" t="n">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="I49" t="n">
-        <v>61</v>
+        <v>153</v>
       </c>
       <c r="J49" t="n">
-        <v>90</v>
+        <v>259</v>
       </c>
       <c r="K49" t="n">
-        <v>169</v>
+        <v>432</v>
       </c>
       <c r="L49" t="n">
-        <v>148</v>
+        <v>480</v>
       </c>
       <c r="M49" t="n">
-        <v>95</v>
+        <v>408</v>
       </c>
       <c r="N49" t="n">
-        <v>49</v>
+        <v>212</v>
       </c>
       <c r="O49" t="n">
-        <v>25</v>
+        <v>134</v>
       </c>
       <c r="P49" t="n">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="Q49" t="n">
-        <v>716</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="Q51" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
     </row>
     <row r="52"/>
@@ -2323,10 +2323,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O55" t="n">
         <v>0</v>
@@ -2344,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -2372,34 +2372,34 @@
         <v>0</v>
       </c>
       <c r="H56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="M56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2733,46 +2733,46 @@
         <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>28</v>
+        <v>94</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>39</v>
+        <v>130</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>50</v>
+        <v>170</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>44</v>
+        <v>156</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>24</v>
+        <v>96</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>22</v>
+        <v>108</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>319</v>
+        <v>1107</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2789,46 +2789,46 @@
         <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F65" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="G65" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="H65" t="n">
-        <v>21</v>
+        <v>102</v>
       </c>
       <c r="I65" t="n">
-        <v>60</v>
+        <v>148</v>
       </c>
       <c r="J65" t="n">
-        <v>83</v>
+        <v>242</v>
       </c>
       <c r="K65" t="n">
-        <v>162</v>
+        <v>409</v>
       </c>
       <c r="L65" t="n">
-        <v>142</v>
+        <v>466</v>
       </c>
       <c r="M65" t="n">
-        <v>93</v>
+        <v>389</v>
       </c>
       <c r="N65" t="n">
-        <v>49</v>
+        <v>206</v>
       </c>
       <c r="O65" t="n">
-        <v>25</v>
+        <v>133</v>
       </c>
       <c r="P65" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="Q65" t="n">
-        <v>684</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="Q67" t="n">
-        <v>15</v>
+        <v>53</v>
       </c>
     </row>
     <row r="68"/>
@@ -3068,10 +3068,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>
@@ -3080,7 +3080,7 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O71" t="n">
         <v>0</v>
@@ -3089,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -3138,13 +3138,13 @@
         <v>0</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3490,19 +3490,19 @@
         <v>0</v>
       </c>
       <c r="H80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J80" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L80" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M80" s="4" t="n">
         <v>1</v>
@@ -3514,10 +3514,10 @@
         <v>0</v>
       </c>
       <c r="P80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q80" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3546,26 +3546,26 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J81" t="n">
+        <v>6</v>
+      </c>
+      <c r="K81" t="n">
+        <v>2</v>
+      </c>
+      <c r="L81" t="n">
+        <v>2</v>
+      </c>
+      <c r="M81" t="n">
+        <v>4</v>
+      </c>
+      <c r="N81" t="n">
         <v>1</v>
       </c>
-      <c r="K81" t="n">
-        <v>0</v>
-      </c>
-      <c r="L81" t="n">
-        <v>1</v>
-      </c>
-      <c r="M81" t="n">
-        <v>0</v>
-      </c>
-      <c r="N81" t="n">
-        <v>0</v>
-      </c>
       <c r="O81" t="n">
         <v>0</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="82"/>
@@ -3687,7 +3687,7 @@
         <v>0</v>
       </c>
       <c r="E85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
@@ -3705,10 +3705,10 @@
         <v>0</v>
       </c>
       <c r="K85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M85" t="n">
         <v>0</v>
@@ -3717,13 +3717,13 @@
         <v>0</v>
       </c>
       <c r="O85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P85" t="n">
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86">
@@ -3739,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="D86" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E86" s="4" t="n">
         <v>0</v>
@@ -3754,16 +3754,16 @@
         <v>0</v>
       </c>
       <c r="I86" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J86" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K86" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L86" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M86" s="4" t="n">
         <v>0</v>
@@ -3772,13 +3772,13 @@
         <v>0</v>
       </c>
       <c r="O86" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P86" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q86" s="4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R86" s="4" t="n"/>
     </row>
@@ -3899,10 +3899,10 @@
         <v>0</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H90" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I90" s="4" t="n">
         <v>0</v>
@@ -3911,14 +3911,14 @@
         <v>1</v>
       </c>
       <c r="K90" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M90" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="N90" s="4" t="n">
         <v>0</v>
       </c>
@@ -3929,7 +3929,7 @@
         <v>0</v>
       </c>
       <c r="Q90" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R90" s="4" t="n"/>
     </row>
@@ -3949,34 +3949,34 @@
         <v>0</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G91" t="n">
+        <v>4</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" t="n">
+        <v>2</v>
+      </c>
+      <c r="J91" t="n">
         <v>1</v>
       </c>
-      <c r="H91" t="n">
-        <v>0</v>
-      </c>
-      <c r="I91" t="n">
-        <v>0</v>
-      </c>
-      <c r="J91" t="n">
-        <v>0</v>
-      </c>
       <c r="K91" t="n">
         <v>0</v>
       </c>
       <c r="L91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O91" t="n">
         <v>0</v>
@@ -3985,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="92"/>
@@ -4093,49 +4093,49 @@
         <v>0</v>
       </c>
       <c r="C95" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F95" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G95" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="H95" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="I95" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="J95" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="K95" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="L95" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="M95" t="n">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="N95" t="n">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="O95" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="P95" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="Q95" t="n">
-        <v>106</v>
+        <v>322</v>
       </c>
     </row>
     <row r="96">
@@ -4148,49 +4148,49 @@
         <v>0</v>
       </c>
       <c r="C96" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D96" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E96" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>22</v>
+        <v>76</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>55</v>
+        <v>128</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>41</v>
+        <v>115</v>
       </c>
       <c r="N96" s="4" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="O96" s="4" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="P96" s="4" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="Q96" s="4" t="n">
-        <v>229</v>
+        <v>656</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
added columns_to_read parameter to loadfile function
</commit_message>
<xml_diff>
--- a/ART MSF SUMMARY AS AT April 2025.xlsx
+++ b/ART MSF SUMMARY AS AT April 2025.xlsx
@@ -464,15 +464,15 @@
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
     <col width="2" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Onitsha General Hospital ART Monthly Summary Form As At April 2025</t>
+          <t>Holy Rosary Hospital ART Monthly Summary Form As At April 2025</t>
         </is>
       </c>
     </row>
@@ -592,10 +592,10 @@
         <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>0</v>
@@ -604,25 +604,25 @@
         <v>1</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="R4" s="4" t="n"/>
     </row>
@@ -642,43 +642,43 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" t="n">
-        <v>4</v>
-      </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
         <v>1</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>3</v>
-      </c>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -733,7 +733,7 @@
         <v/>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" s="4" t="n"/>
     </row>
@@ -953,49 +953,49 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I12" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>106</v>
-      </c>
       <c r="J12" s="4" t="n">
-        <v>134</v>
+        <v>41</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>154</v>
+        <v>75</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>216</v>
+        <v>64</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>189</v>
+        <v>56</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>107</v>
+        <v>27</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1425</v>
+        <v>411</v>
       </c>
       <c r="R12" s="4" t="n"/>
     </row>
@@ -1012,46 +1012,46 @@
         <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="H13" t="n">
-        <v>134</v>
+        <v>31</v>
       </c>
       <c r="I13" t="n">
-        <v>191</v>
+        <v>71</v>
       </c>
       <c r="J13" t="n">
-        <v>314</v>
+        <v>104</v>
       </c>
       <c r="K13" t="n">
-        <v>524</v>
+        <v>197</v>
       </c>
       <c r="L13" t="n">
-        <v>560</v>
+        <v>178</v>
       </c>
       <c r="M13" t="n">
-        <v>469</v>
+        <v>113</v>
       </c>
       <c r="N13" t="n">
-        <v>247</v>
+        <v>55</v>
       </c>
       <c r="O13" t="n">
-        <v>146</v>
+        <v>28</v>
       </c>
       <c r="P13" t="n">
-        <v>138</v>
+        <v>29</v>
       </c>
       <c r="Q13" t="n">
-        <v>2877</v>
+        <v>847</v>
       </c>
     </row>
     <row r="14">
@@ -1106,7 +1106,7 @@
         <v/>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="R14" s="4" t="n"/>
     </row>
@@ -1162,7 +1162,7 @@
         <v/>
       </c>
       <c r="Q15" t="n">
-        <v>65</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16"/>
@@ -1207,16 +1207,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C19" t="n">
-        <v>1369</v>
+        <v>400</v>
       </c>
       <c r="D19" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
-        <v>2803</v>
+        <v>838</v>
       </c>
     </row>
     <row r="20">
@@ -1229,13 +1229,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F20" s="4" t="n"/>
     </row>
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1390</v>
+        <v>400</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>2835</v>
+        <v>838</v>
       </c>
       <c r="F22" s="4" t="n"/>
     </row>
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>752</v>
+        <v>298</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1573</v>
+        <v>644</v>
       </c>
       <c r="F26" s="4" t="n"/>
     </row>
@@ -1343,13 +1343,13 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1379,16 +1379,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>443</v>
+        <v>98</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>952</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30">
@@ -1398,16 +1398,16 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1235</v>
+        <v>396</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>2594</v>
+        <v>831</v>
       </c>
       <c r="F30" s="4" t="n"/>
     </row>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>4002</v>
+        <v>1250</v>
       </c>
       <c r="C34" s="4" t="n"/>
     </row>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>129</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36"/>
@@ -1572,22 +1572,22 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N39" t="n">
         <v>0</v>
@@ -1596,10 +1596,10 @@
         <v>0</v>
       </c>
       <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
         <v>2</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -1630,31 +1630,31 @@
         <v>0</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q40" s="4" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="R40" s="4" t="n"/>
     </row>
@@ -1710,7 +1710,7 @@
         <v/>
       </c>
       <c r="Q41" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -1765,7 +1765,7 @@
         <v/>
       </c>
       <c r="Q42" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R42" s="4" t="n"/>
     </row>
@@ -1821,7 +1821,7 @@
         <v/>
       </c>
       <c r="Q43" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44">
@@ -1876,7 +1876,7 @@
         <v/>
       </c>
       <c r="Q44" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R44" s="4" t="n"/>
     </row>
@@ -1985,49 +1985,49 @@
         <v>0</v>
       </c>
       <c r="C48" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>103</v>
+        <v>33</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>140</v>
+        <v>41</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>130</v>
+        <v>64</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>180</v>
+        <v>52</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>166</v>
+        <v>45</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="P48" s="4" t="n">
-        <v>112</v>
+        <v>23</v>
       </c>
       <c r="Q48" s="4" t="n">
-        <v>1184</v>
+        <v>344</v>
       </c>
       <c r="R48" s="4" t="n"/>
     </row>
@@ -2041,49 +2041,49 @@
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="n">
         <v>11</v>
       </c>
-      <c r="E49" t="n">
-        <v>19</v>
-      </c>
-      <c r="F49" t="n">
-        <v>28</v>
-      </c>
       <c r="G49" t="n">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="H49" t="n">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="I49" t="n">
-        <v>153</v>
+        <v>61</v>
       </c>
       <c r="J49" t="n">
-        <v>259</v>
+        <v>90</v>
       </c>
       <c r="K49" t="n">
-        <v>432</v>
+        <v>169</v>
       </c>
       <c r="L49" t="n">
-        <v>480</v>
+        <v>148</v>
       </c>
       <c r="M49" t="n">
-        <v>408</v>
+        <v>95</v>
       </c>
       <c r="N49" t="n">
-        <v>212</v>
+        <v>49</v>
       </c>
       <c r="O49" t="n">
-        <v>134</v>
+        <v>25</v>
       </c>
       <c r="P49" t="n">
-        <v>120</v>
+        <v>24</v>
       </c>
       <c r="Q49" t="n">
-        <v>2418</v>
+        <v>716</v>
       </c>
     </row>
     <row r="50">
@@ -2138,7 +2138,7 @@
         <v/>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="R50" s="4" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="Q51" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52"/>
@@ -2323,10 +2323,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
@@ -2335,7 +2335,7 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O55" t="n">
         <v>0</v>
@@ -2344,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56">
@@ -2372,11 +2372,11 @@
         <v>0</v>
       </c>
       <c r="H56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I56" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J56" s="4" t="n">
         <v>0</v>
       </c>
@@ -2384,22 +2384,22 @@
         <v>0</v>
       </c>
       <c r="L56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M56" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="N56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P56" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q56" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R56" s="4" t="n"/>
     </row>
@@ -2733,46 +2733,46 @@
         <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>130</v>
+        <v>39</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>170</v>
+        <v>50</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="O64" s="4" t="n">
-        <v>96</v>
+        <v>24</v>
       </c>
       <c r="P64" s="4" t="n">
-        <v>108</v>
+        <v>22</v>
       </c>
       <c r="Q64" s="4" t="n">
-        <v>1107</v>
+        <v>319</v>
       </c>
       <c r="R64" s="4" t="n"/>
     </row>
@@ -2789,46 +2789,46 @@
         <v>2</v>
       </c>
       <c r="D65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" t="n">
+        <v>8</v>
+      </c>
+      <c r="G65" t="n">
         <v>11</v>
       </c>
-      <c r="E65" t="n">
-        <v>19</v>
-      </c>
-      <c r="F65" t="n">
-        <v>27</v>
-      </c>
-      <c r="G65" t="n">
-        <v>43</v>
-      </c>
       <c r="H65" t="n">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="I65" t="n">
-        <v>148</v>
+        <v>60</v>
       </c>
       <c r="J65" t="n">
-        <v>242</v>
+        <v>83</v>
       </c>
       <c r="K65" t="n">
-        <v>409</v>
+        <v>162</v>
       </c>
       <c r="L65" t="n">
-        <v>466</v>
+        <v>142</v>
       </c>
       <c r="M65" t="n">
-        <v>389</v>
+        <v>93</v>
       </c>
       <c r="N65" t="n">
-        <v>206</v>
+        <v>49</v>
       </c>
       <c r="O65" t="n">
-        <v>133</v>
+        <v>25</v>
       </c>
       <c r="P65" t="n">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="Q65" t="n">
-        <v>2313</v>
+        <v>684</v>
       </c>
     </row>
     <row r="66">
@@ -2883,7 +2883,7 @@
         <v/>
       </c>
       <c r="Q66" s="4" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="R66" s="4" t="n"/>
     </row>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="Q67" t="n">
-        <v>53</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68"/>
@@ -3068,10 +3068,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>
@@ -3080,7 +3080,7 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O71" t="n">
         <v>0</v>
@@ -3089,7 +3089,7 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
@@ -3138,13 +3138,13 @@
         <v>0</v>
       </c>
       <c r="O72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P72" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R72" s="4" t="n"/>
     </row>
@@ -3490,19 +3490,19 @@
         <v>0</v>
       </c>
       <c r="H80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I80" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J80" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L80" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M80" s="4" t="n">
         <v>1</v>
@@ -3514,10 +3514,10 @@
         <v>0</v>
       </c>
       <c r="P80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="Q80" s="4" t="n">
-        <v>11</v>
       </c>
       <c r="R80" s="4" t="n"/>
     </row>
@@ -3546,34 +3546,34 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
         <v>1</v>
       </c>
-      <c r="I81" t="n">
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
         <v>2</v>
-      </c>
-      <c r="J81" t="n">
-        <v>6</v>
-      </c>
-      <c r="K81" t="n">
-        <v>2</v>
-      </c>
-      <c r="L81" t="n">
-        <v>2</v>
-      </c>
-      <c r="M81" t="n">
-        <v>4</v>
-      </c>
-      <c r="N81" t="n">
-        <v>1</v>
-      </c>
-      <c r="O81" t="n">
-        <v>0</v>
-      </c>
-      <c r="P81" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q81" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="82"/>
@@ -3687,7 +3687,7 @@
         <v>0</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
@@ -3705,10 +3705,10 @@
         <v>0</v>
       </c>
       <c r="K85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M85" t="n">
         <v>0</v>
@@ -3717,13 +3717,13 @@
         <v>0</v>
       </c>
       <c r="O85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P85" t="n">
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3739,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="D86" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E86" s="4" t="n">
         <v>0</v>
@@ -3754,16 +3754,16 @@
         <v>0</v>
       </c>
       <c r="I86" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J86" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K86" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L86" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M86" s="4" t="n">
         <v>0</v>
@@ -3772,13 +3772,13 @@
         <v>0</v>
       </c>
       <c r="O86" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P86" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q86" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R86" s="4" t="n"/>
     </row>
@@ -3899,10 +3899,10 @@
         <v>0</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H90" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I90" s="4" t="n">
         <v>0</v>
@@ -3911,25 +3911,25 @@
         <v>1</v>
       </c>
       <c r="K90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="L90" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M90" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N90" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O90" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P90" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q90" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="R90" s="4" t="n"/>
     </row>
@@ -3949,43 +3949,43 @@
         <v>0</v>
       </c>
       <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
         <v>1</v>
       </c>
-      <c r="F91" t="n">
-        <v>3</v>
-      </c>
-      <c r="G91" t="n">
-        <v>4</v>
-      </c>
       <c r="H91" t="n">
         <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="n">
         <v>1</v>
-      </c>
-      <c r="K91" t="n">
-        <v>0</v>
-      </c>
-      <c r="L91" t="n">
-        <v>3</v>
-      </c>
-      <c r="M91" t="n">
-        <v>1</v>
-      </c>
-      <c r="N91" t="n">
-        <v>1</v>
-      </c>
-      <c r="O91" t="n">
-        <v>0</v>
-      </c>
-      <c r="P91" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q91" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="92"/>
@@ -4093,49 +4093,49 @@
         <v>0</v>
       </c>
       <c r="C95" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
         <v>2</v>
       </c>
-      <c r="D95" t="n">
-        <v>4</v>
-      </c>
-      <c r="E95" t="n">
-        <v>10</v>
-      </c>
       <c r="F95" t="n">
+        <v>5</v>
+      </c>
+      <c r="G95" t="n">
+        <v>5</v>
+      </c>
+      <c r="H95" t="n">
+        <v>3</v>
+      </c>
+      <c r="I95" t="n">
+        <v>6</v>
+      </c>
+      <c r="J95" t="n">
+        <v>11</v>
+      </c>
+      <c r="K95" t="n">
         <v>13</v>
       </c>
-      <c r="G95" t="n">
+      <c r="L95" t="n">
         <v>20</v>
       </c>
-      <c r="H95" t="n">
-        <v>21</v>
-      </c>
-      <c r="I95" t="n">
-        <v>25</v>
-      </c>
-      <c r="J95" t="n">
-        <v>33</v>
-      </c>
-      <c r="K95" t="n">
-        <v>42</v>
-      </c>
-      <c r="L95" t="n">
-        <v>32</v>
-      </c>
       <c r="M95" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="N95" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="O95" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="P95" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="Q95" t="n">
-        <v>322</v>
+        <v>106</v>
       </c>
     </row>
     <row r="96">
@@ -4148,49 +4148,49 @@
         <v>0</v>
       </c>
       <c r="C96" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E96" s="4" t="n">
+      <c r="G96" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H96" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F96" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G96" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H96" s="4" t="n">
-        <v>32</v>
-      </c>
       <c r="I96" s="4" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>76</v>
+        <v>22</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>128</v>
+        <v>55</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>100</v>
+        <v>47</v>
       </c>
       <c r="M96" s="4" t="n">
-        <v>115</v>
+        <v>41</v>
       </c>
       <c r="N96" s="4" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="O96" s="4" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="P96" s="4" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="Q96" s="4" t="n">
-        <v>656</v>
+        <v>229</v>
       </c>
       <c r="R96" s="4" t="n"/>
     </row>

</xml_diff>